<commit_message>
📝 docs(analysis): TPS, Mean Latency, 95th percentile 취합 완료 #10
</commit_message>
<xml_diff>
--- a/docs/result/analysis/enrollment-burst-test-pessimistic-lock-result.xlsx
+++ b/docs/result/analysis/enrollment-burst-test-pessimistic-lock-result.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sangja/Projects/concurrency-control-benchmarks/docs/result/analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECBE8505-0821-0C41-AC71-7582AC16D3DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA977A7A-30DF-7944-BD72-9FA2609711FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="25600" windowHeight="28200" activeTab="1" xr2:uid="{829354C8-DEED-BD4A-88FD-415D5A61907D}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="2" xr2:uid="{829354C8-DEED-BD4A-88FD-415D5A61907D}"/>
   </bookViews>
   <sheets>
     <sheet name="Pessimistic Lock" sheetId="1" r:id="rId1"/>
     <sheet name="TPS" sheetId="2" r:id="rId2"/>
+    <sheet name="Mean Latency" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="25">
   <si>
     <t>TPS (request/sec)</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -67,11 +68,75 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>평균 TPS</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Vuser</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mean TPS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Peek TPS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Worst Mean TPS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Overall Mean TPS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Best Mean TPS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Average Peak TPS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>취합 TPS (request/sec)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mean Latency (ms)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Mean Latency</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>취합 Mean Latency (ms)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Worst Mean Latency</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Overall Mean Latency</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Best Mean Latency</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>95th Percentile (추정치)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Worst 95th Percentile</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Overall 95th Percentile</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Best 95th Percentile</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -469,136 +534,697 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6CE196A4-CB6E-9740-BA12-8F5D37C430EC}">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:L18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.7109375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:12">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
-    </row>
-    <row r="2" spans="1:3">
+      <c r="D1" s="1"/>
+      <c r="H1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+    </row>
+    <row r="2" spans="1:12">
       <c r="A2" s="1"/>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
-    </row>
-    <row r="3" spans="1:3">
+      <c r="D2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" t="s">
         <v>6</v>
       </c>
       <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:3">
+      <c r="I3" t="s">
+        <v>10</v>
+      </c>
+      <c r="J3" t="s">
+        <v>11</v>
+      </c>
+      <c r="K3" t="s">
+        <v>12</v>
+      </c>
+      <c r="L3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B4">
         <v>500</v>
       </c>
-    </row>
-    <row r="5" spans="1:3">
+      <c r="C4">
+        <v>41.5</v>
+      </c>
+      <c r="D4">
+        <v>107</v>
+      </c>
+      <c r="H4">
+        <v>500</v>
+      </c>
+      <c r="I4">
+        <f>MIN(C4,C7,C10,C13,C16)</f>
+        <v>35.6</v>
+      </c>
+      <c r="J4">
+        <f>AVERAGE(C4,C7,C10,C13,C16)</f>
+        <v>50.3</v>
+      </c>
+      <c r="K4">
+        <f>MAX(C4,C7,C10,C13,C16)</f>
+        <v>62.3</v>
+      </c>
+      <c r="L4">
+        <f>AVERAGE(D4,D7,D10,D13,D16)</f>
+        <v>125.8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" s="1"/>
       <c r="B5">
         <v>800</v>
       </c>
-    </row>
-    <row r="6" spans="1:3">
+      <c r="C5">
+        <v>99.7</v>
+      </c>
+      <c r="D5">
+        <v>243</v>
+      </c>
+      <c r="H5">
+        <v>800</v>
+      </c>
+      <c r="I5">
+        <f>MIN(C5,C8,C11,C14,C17)</f>
+        <v>66.3</v>
+      </c>
+      <c r="J5">
+        <f>AVERAGE(C5,C8,C11,C14,C17)</f>
+        <v>82.34</v>
+      </c>
+      <c r="K5">
+        <f>MAX(C5,C8,C11,C14,C17)</f>
+        <v>99.7</v>
+      </c>
+      <c r="L5">
+        <f>AVERAGE(D5,D8,D11,D14,D17)</f>
+        <v>214.7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6" s="1"/>
       <c r="B6">
         <v>1000</v>
       </c>
-    </row>
-    <row r="7" spans="1:3">
+      <c r="C6">
+        <v>62.3</v>
+      </c>
+      <c r="D6">
+        <v>207</v>
+      </c>
+      <c r="H6">
+        <v>1000</v>
+      </c>
+      <c r="I6">
+        <f>MIN(C6,C9,C12,C15,C18)</f>
+        <v>62.3</v>
+      </c>
+      <c r="J6">
+        <f>AVERAGE(C6,C9,C12,C15,C18)</f>
+        <v>85.47999999999999</v>
+      </c>
+      <c r="K6">
+        <f>MAX(C6,C9,C12,C15,C18)</f>
+        <v>99.6</v>
+      </c>
+      <c r="L6">
+        <f>AVERAGE(D6,D9,D12,D15,D18)</f>
+        <v>189.2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B7">
         <v>500</v>
       </c>
-    </row>
-    <row r="8" spans="1:3">
+      <c r="C7">
+        <v>49.8</v>
+      </c>
+      <c r="D7">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="8" spans="1:12">
       <c r="A8" s="1"/>
       <c r="B8">
         <v>800</v>
       </c>
-    </row>
-    <row r="9" spans="1:3">
+      <c r="C8">
+        <v>79.8</v>
+      </c>
+      <c r="D8">
+        <v>228.5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12">
       <c r="A9" s="1"/>
       <c r="B9">
         <v>1000</v>
       </c>
-    </row>
-    <row r="10" spans="1:3">
+      <c r="C9">
+        <v>99.5</v>
+      </c>
+      <c r="D9">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="10" spans="1:12">
       <c r="A10" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B10">
         <v>500</v>
       </c>
-    </row>
-    <row r="11" spans="1:3">
+      <c r="C10">
+        <v>62.3</v>
+      </c>
+      <c r="D10">
+        <v>139.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:12">
       <c r="A11" s="1"/>
       <c r="B11">
         <v>800</v>
       </c>
-    </row>
-    <row r="12" spans="1:3">
+      <c r="C11">
+        <v>66.3</v>
+      </c>
+      <c r="D11">
+        <v>192.5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12" s="1"/>
       <c r="B12">
         <v>1000</v>
       </c>
-    </row>
-    <row r="13" spans="1:3">
+      <c r="C12">
+        <v>83</v>
+      </c>
+      <c r="D12">
+        <v>150.5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:12">
       <c r="A13" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B13">
         <v>500</v>
       </c>
-    </row>
-    <row r="14" spans="1:3">
+      <c r="C13">
+        <v>35.6</v>
+      </c>
+      <c r="D13">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="14" spans="1:12">
       <c r="A14" s="1"/>
       <c r="B14">
         <v>800</v>
       </c>
-    </row>
-    <row r="15" spans="1:3">
+      <c r="C14">
+        <v>99.5</v>
+      </c>
+      <c r="D14">
+        <v>285.5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:12">
       <c r="A15" s="1"/>
       <c r="B15">
         <v>1000</v>
       </c>
-    </row>
-    <row r="16" spans="1:3">
+      <c r="C15">
+        <v>99.6</v>
+      </c>
+      <c r="D15">
+        <v>241.5</v>
+      </c>
+    </row>
+    <row r="16" spans="1:12">
       <c r="A16" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B16">
         <v>500</v>
       </c>
-    </row>
-    <row r="17" spans="1:2">
+      <c r="C16">
+        <v>62.3</v>
+      </c>
+      <c r="D16">
+        <v>170.5</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
       <c r="A17" s="1"/>
       <c r="B17">
         <v>800</v>
       </c>
-    </row>
-    <row r="18" spans="1:2">
+      <c r="C17">
+        <v>66.400000000000006</v>
+      </c>
+      <c r="D17">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
       <c r="A18" s="1"/>
       <c r="B18">
         <v>1000</v>
       </c>
+      <c r="C18">
+        <v>83</v>
+      </c>
+      <c r="D18">
+        <v>146</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
+    <mergeCell ref="H1:L2"/>
     <mergeCell ref="A16:A18"/>
-    <mergeCell ref="A1:C2"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="A13:A15"/>
+    <mergeCell ref="A1:D2"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{50C2AED8-BFB4-1946-BD50-4033FDA20FC9}">
+  <dimension ref="A1:N18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" customWidth="1"/>
+    <col min="4" max="4" width="20.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="H1" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" t="s">
+        <v>18</v>
+      </c>
+      <c r="J3" t="s">
+        <v>19</v>
+      </c>
+      <c r="K3" t="s">
+        <v>20</v>
+      </c>
+      <c r="L3" t="s">
+        <v>22</v>
+      </c>
+      <c r="M3" t="s">
+        <v>23</v>
+      </c>
+      <c r="N3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>500</v>
+      </c>
+      <c r="C4">
+        <v>521.95000000000005</v>
+      </c>
+      <c r="D4">
+        <v>1260.73</v>
+      </c>
+      <c r="H4">
+        <v>500</v>
+      </c>
+      <c r="I4">
+        <f>MAX(C4,C7,C10,C13,C16)</f>
+        <v>732.61</v>
+      </c>
+      <c r="J4">
+        <f>AVERAGE(C4,C7,C10,C13,C16)</f>
+        <v>556.57800000000009</v>
+      </c>
+      <c r="K4">
+        <f>MIN(C4,C7,C10,C13,C16)</f>
+        <v>409.65</v>
+      </c>
+      <c r="L4">
+        <f>MAX(D4,D7,D10,D13,D16)</f>
+        <v>1671.6</v>
+      </c>
+      <c r="M4">
+        <f>AVERAGE(D4,D7,D10,D13,D16)</f>
+        <v>1300.69</v>
+      </c>
+      <c r="N4">
+        <f>MIN(D4,D7,D10,D13,D16)</f>
+        <v>987.85</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" s="1"/>
+      <c r="B5">
+        <v>800</v>
+      </c>
+      <c r="C5">
+        <v>1176.68</v>
+      </c>
+      <c r="D5">
+        <v>2299.5</v>
+      </c>
+      <c r="H5">
+        <v>800</v>
+      </c>
+      <c r="I5">
+        <f>MAX(C5,C8,C11,C14,C17)</f>
+        <v>1303.32</v>
+      </c>
+      <c r="J5">
+        <f>AVERAGE(C5,C8,C11,C14,C17)</f>
+        <v>1041.7339999999999</v>
+      </c>
+      <c r="K5">
+        <f>MIN(C5,C8,C11,C14,C17)</f>
+        <v>828.86</v>
+      </c>
+      <c r="L5">
+        <f>MAX(D5,D8,D11,D14,D17)</f>
+        <v>2410.56</v>
+      </c>
+      <c r="M5">
+        <f>AVERAGE(D5,D8,D11,D14,D17)</f>
+        <v>1999.2380000000001</v>
+      </c>
+      <c r="N5">
+        <f>MIN(D5,D8,D11,D14,D17)</f>
+        <v>1623.93</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="1"/>
+      <c r="B6">
+        <v>1000</v>
+      </c>
+      <c r="C6">
+        <v>1065.08</v>
+      </c>
+      <c r="D6">
+        <v>2212.87</v>
+      </c>
+      <c r="H6">
+        <v>1000</v>
+      </c>
+      <c r="I6">
+        <f>MAX(C6,C9,C12,C15,C18)</f>
+        <v>1124.9100000000001</v>
+      </c>
+      <c r="J6">
+        <f>AVERAGE(C6,C9,C12,C15,C18)</f>
+        <v>1012.8899999999998</v>
+      </c>
+      <c r="K6">
+        <f>MIN(C6,C9,C12,C15,C18)</f>
+        <v>764.98</v>
+      </c>
+      <c r="L6">
+        <f>MAX(D6,D9,D12,D15,D18)</f>
+        <v>2275.0100000000002</v>
+      </c>
+      <c r="M6">
+        <f>AVERAGE(D6,D9,D12,D15,D18)</f>
+        <v>2093.9360000000001</v>
+      </c>
+      <c r="N6">
+        <f>MIN(D6,D9,D12,D15,D18)</f>
+        <v>1674.41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7">
+        <v>500</v>
+      </c>
+      <c r="C7">
+        <v>448.85</v>
+      </c>
+      <c r="D7">
+        <v>1168.73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" s="1"/>
+      <c r="B8">
+        <v>800</v>
+      </c>
+      <c r="C8">
+        <v>828.86</v>
+      </c>
+      <c r="D8">
+        <v>1623.93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" s="1"/>
+      <c r="B9">
+        <v>1000</v>
+      </c>
+      <c r="C9">
+        <v>1124.9100000000001</v>
+      </c>
+      <c r="D9">
+        <v>2275.0100000000002</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>500</v>
+      </c>
+      <c r="C10">
+        <v>669.83</v>
+      </c>
+      <c r="D10">
+        <v>1414.54</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" s="1"/>
+      <c r="B11">
+        <v>800</v>
+      </c>
+      <c r="C11">
+        <v>1028.52</v>
+      </c>
+      <c r="D11">
+        <v>1873.72</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" s="1"/>
+      <c r="B12">
+        <v>1000</v>
+      </c>
+      <c r="C12">
+        <v>1069.21</v>
+      </c>
+      <c r="D12">
+        <v>2170.84</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13">
+        <v>500</v>
+      </c>
+      <c r="C13">
+        <v>409.65</v>
+      </c>
+      <c r="D13">
+        <v>987.85</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" s="1"/>
+      <c r="B14">
+        <v>800</v>
+      </c>
+      <c r="C14">
+        <v>1303.32</v>
+      </c>
+      <c r="D14">
+        <v>2410.56</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" s="1"/>
+      <c r="B15">
+        <v>1000</v>
+      </c>
+      <c r="C15">
+        <v>1040.27</v>
+      </c>
+      <c r="D15">
+        <v>2136.5500000000002</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16">
+        <v>500</v>
+      </c>
+      <c r="C16">
+        <v>732.61</v>
+      </c>
+      <c r="D16">
+        <v>1671.6</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4">
+      <c r="A17" s="1"/>
+      <c r="B17">
+        <v>800</v>
+      </c>
+      <c r="C17">
+        <v>871.29</v>
+      </c>
+      <c r="D17">
+        <v>1788.48</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4">
+      <c r="A18" s="1"/>
+      <c r="B18">
+        <v>1000</v>
+      </c>
+      <c r="C18">
+        <f>764.98</f>
+        <v>764.98</v>
+      </c>
+      <c r="D18">
+        <v>1674.41</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A1:D2"/>
+    <mergeCell ref="H1:N2"/>
+    <mergeCell ref="A16:A18"/>
     <mergeCell ref="A4:A6"/>
     <mergeCell ref="A7:A9"/>
     <mergeCell ref="A10:A12"/>

</xml_diff>

<commit_message>
📝 docs(analysis): 안정성 취합중 #10
</commit_message>
<xml_diff>
--- a/docs/result/analysis/enrollment-burst-test-pessimistic-lock-result.xlsx
+++ b/docs/result/analysis/enrollment-burst-test-pessimistic-lock-result.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/sangja/Projects/concurrency-control-benchmarks/docs/result/analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA977A7A-30DF-7944-BD72-9FA2609711FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD181165-80F0-8B48-984C-9BB99CA46134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" activeTab="2" xr2:uid="{829354C8-DEED-BD4A-88FD-415D5A61907D}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="14700" windowHeight="18460" activeTab="3" xr2:uid="{829354C8-DEED-BD4A-88FD-415D5A61907D}"/>
   </bookViews>
   <sheets>
     <sheet name="Pessimistic Lock" sheetId="1" r:id="rId1"/>
     <sheet name="TPS" sheetId="2" r:id="rId2"/>
     <sheet name="Mean Latency" sheetId="3" r:id="rId3"/>
+    <sheet name="안정성" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="29">
   <si>
     <t>TPS (request/sec)</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -76,10 +77,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>Peek TPS</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Worst Mean TPS</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -137,6 +134,26 @@
   </si>
   <si>
     <t>Best 95th Percentile</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Peak TPS</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>표준편차(σ)</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>아키텍처 안정성</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2σ 변동폭</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>취합 아키텍처 안정성 (ms)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -556,7 +573,7 @@
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="H1" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
@@ -585,22 +602,22 @@
         <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="H3" t="s">
         <v>7</v>
       </c>
       <c r="I3" t="s">
+        <v>9</v>
+      </c>
+      <c r="J3" t="s">
         <v>10</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>11</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>12</v>
-      </c>
-      <c r="L3" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="4" spans="1:12">
@@ -885,13 +902,13 @@
   <sheetData>
     <row r="1" spans="1:14">
       <c r="A1" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
       <c r="H1" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
@@ -921,31 +938,31 @@
         <v>7</v>
       </c>
       <c r="C3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="D3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H3" t="s">
         <v>7</v>
       </c>
       <c r="I3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" t="s">
         <v>18</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>19</v>
       </c>
-      <c r="K3" t="s">
-        <v>20</v>
-      </c>
       <c r="L3" t="s">
+        <v>21</v>
+      </c>
+      <c r="M3" t="s">
         <v>22</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>23</v>
-      </c>
-      <c r="N3" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:14">
@@ -1233,4 +1250,382 @@
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A219465C-BD8C-C648-AF31-5540E51E89B7}">
+  <dimension ref="A1:N18"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="18"/>
+  <cols>
+    <col min="1" max="1" width="6.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.42578125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
+      <c r="H1" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I1" s="1"/>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>15</v>
+      </c>
+      <c r="D3" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" t="s">
+        <v>17</v>
+      </c>
+      <c r="J3" t="s">
+        <v>18</v>
+      </c>
+      <c r="K3" t="s">
+        <v>19</v>
+      </c>
+      <c r="L3" t="s">
+        <v>21</v>
+      </c>
+      <c r="M3" t="s">
+        <v>22</v>
+      </c>
+      <c r="N3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14">
+      <c r="A4" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B4">
+        <v>500</v>
+      </c>
+      <c r="C4">
+        <v>521.95000000000005</v>
+      </c>
+      <c r="D4">
+        <v>395.96</v>
+      </c>
+      <c r="E4">
+        <v>791.93</v>
+      </c>
+      <c r="H4">
+        <v>500</v>
+      </c>
+      <c r="I4">
+        <f>MAX(C4,C7,C10,C13,C16)</f>
+        <v>732.61</v>
+      </c>
+      <c r="J4">
+        <f>AVERAGE(C4,C7,C10,C13,C16)</f>
+        <v>556.57800000000009</v>
+      </c>
+      <c r="K4">
+        <f>MIN(C4,C7,C10,C13,C16)</f>
+        <v>409.65</v>
+      </c>
+      <c r="L4">
+        <f>MAX(D4,D7,D10,D13,D16)</f>
+        <v>395.96</v>
+      </c>
+      <c r="M4">
+        <f>AVERAGE(D4,D7,D10,D13,D16)</f>
+        <v>394.24666666666667</v>
+      </c>
+      <c r="N4">
+        <f>MIN(D4,D7,D10,D13,D16)</f>
+        <v>393.3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14">
+      <c r="A5" s="1"/>
+      <c r="B5">
+        <v>800</v>
+      </c>
+      <c r="C5">
+        <v>1176.68</v>
+      </c>
+      <c r="D5">
+        <v>593.29999999999995</v>
+      </c>
+      <c r="E5">
+        <v>1186.5999999999999</v>
+      </c>
+      <c r="H5">
+        <v>800</v>
+      </c>
+      <c r="I5">
+        <f>MAX(C5,C8,C11,C14,C17)</f>
+        <v>1303.32</v>
+      </c>
+      <c r="J5">
+        <f>AVERAGE(C5,C8,C11,C14,C17)</f>
+        <v>1041.7339999999999</v>
+      </c>
+      <c r="K5">
+        <f>MIN(C5,C8,C11,C14,C17)</f>
+        <v>828.86</v>
+      </c>
+      <c r="L5">
+        <f>MAX(D5,D8,D11,D14,D17)</f>
+        <v>593.29999999999995</v>
+      </c>
+      <c r="M5">
+        <f>AVERAGE(D5,D8,D11,D14,D17)</f>
+        <v>487.31333333333333</v>
+      </c>
+      <c r="N5">
+        <f>MIN(D5,D8,D11,D14,D17)</f>
+        <v>420.03</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="1"/>
+      <c r="B6">
+        <v>1000</v>
+      </c>
+      <c r="C6">
+        <v>1065.08</v>
+      </c>
+      <c r="D6">
+        <v>605.86</v>
+      </c>
+      <c r="E6">
+        <v>1211.73</v>
+      </c>
+      <c r="H6">
+        <v>1000</v>
+      </c>
+      <c r="I6">
+        <f>MAX(C6,C9,C12,C15,C18)</f>
+        <v>1124.9100000000001</v>
+      </c>
+      <c r="J6">
+        <f>AVERAGE(C6,C9,C12,C15,C18)</f>
+        <v>1012.8899999999998</v>
+      </c>
+      <c r="K6">
+        <f>MIN(C6,C9,C12,C15,C18)</f>
+        <v>764.98</v>
+      </c>
+      <c r="L6">
+        <f>MAX(D6,D9,D12,D15,D18)</f>
+        <v>607.25</v>
+      </c>
+      <c r="M6">
+        <f>AVERAGE(D6,D9,D12,D15,D18)</f>
+        <v>598.19333333333338</v>
+      </c>
+      <c r="N6">
+        <f>MIN(D6,D9,D12,D15,D18)</f>
+        <v>581.47</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14">
+      <c r="A7" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7">
+        <v>500</v>
+      </c>
+      <c r="C7">
+        <v>448.85</v>
+      </c>
+      <c r="D7">
+        <v>393.48</v>
+      </c>
+      <c r="E7">
+        <v>786.96</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14">
+      <c r="A8" s="1"/>
+      <c r="B8">
+        <v>800</v>
+      </c>
+      <c r="C8">
+        <v>828.86</v>
+      </c>
+      <c r="D8">
+        <v>420.03</v>
+      </c>
+      <c r="E8">
+        <v>840.06</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14">
+      <c r="A9" s="1"/>
+      <c r="B9">
+        <v>1000</v>
+      </c>
+      <c r="C9">
+        <v>1124.9100000000001</v>
+      </c>
+      <c r="D9">
+        <v>607.25</v>
+      </c>
+      <c r="E9">
+        <v>1214.49</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14">
+      <c r="A10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10">
+        <v>500</v>
+      </c>
+      <c r="C10">
+        <v>669.83</v>
+      </c>
+      <c r="D10">
+        <v>393.3</v>
+      </c>
+      <c r="E10">
+        <v>786.59</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14">
+      <c r="A11" s="1"/>
+      <c r="B11">
+        <v>800</v>
+      </c>
+      <c r="C11">
+        <v>1028.52</v>
+      </c>
+      <c r="D11">
+        <v>448.61</v>
+      </c>
+      <c r="E11">
+        <v>897.21</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14">
+      <c r="A12" s="1"/>
+      <c r="B12">
+        <v>1000</v>
+      </c>
+      <c r="C12">
+        <v>1069.21</v>
+      </c>
+      <c r="D12">
+        <v>581.47</v>
+      </c>
+      <c r="E12">
+        <v>1162.94</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14">
+      <c r="A13" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13">
+        <v>500</v>
+      </c>
+      <c r="C13">
+        <v>409.65</v>
+      </c>
+    </row>
+    <row r="14" spans="1:14">
+      <c r="A14" s="1"/>
+      <c r="B14">
+        <v>800</v>
+      </c>
+      <c r="C14">
+        <v>1303.32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:14">
+      <c r="A15" s="1"/>
+      <c r="B15">
+        <v>1000</v>
+      </c>
+      <c r="C15">
+        <v>1040.27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:14">
+      <c r="A16" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B16">
+        <v>500</v>
+      </c>
+      <c r="C16">
+        <v>732.61</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" s="1"/>
+      <c r="B17">
+        <v>800</v>
+      </c>
+      <c r="C17">
+        <v>871.29</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" s="1"/>
+      <c r="B18">
+        <v>1000</v>
+      </c>
+      <c r="C18">
+        <f>764.98</f>
+        <v>764.98</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="A16:A18"/>
+    <mergeCell ref="A1:E2"/>
+    <mergeCell ref="H1:N2"/>
+    <mergeCell ref="A4:A6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="A13:A15"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>